<commit_message>
Add 2006-2026 search: additional SE Asian peat WTD sites and datasets
- EXPANDED_2006-2026.md/.xlsx: 67 sites/datasets not in INDEX.md (8 public,
  9 networks/on request, 44 paper-only, 6 compilations/products), the 87 SE
  Asian water-level sites from Apers et al. 2022 Table B1, and updates to
  existing entries; nothing downloaded
- build_expanded.py regenerates the tables
- DATA_SUMMARY: A8 Acacia coordinate confirmed by Deshmukh et al. 2020;
  A6 note points to public 2011-2014 daily WT for the same forest

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZEc9uEk27URkV1sWwrTAd
</commit_message>
<xml_diff>
--- a/literature/DATA_SUMMARY.xlsx
+++ b/literature/DATA_SUMMARY.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files'!$A$1:$S$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datasets'!$A$1:$H$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data availability'!$A$1:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Corrections'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Corrections'!$A$1:$D$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5889,7 +5889,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>FLUXNET-CH4 covers only 2014-2015 for MY-MLM, not the 2011-2014 period of Tang 2020; the full record is held by the Sarawak Tropical Peat Research Institute. | FLUXNET site metadata: 1.4536, 111.1495, AsiaFlux, EBF. C7 (Aeries 2023) has 2011-2015 water-table loggers in the same national park.</t>
+          <t>FLUXNET-CH4 covers only 2014-2015 for MY-MLM, not the 2011-2014 period of Tang 2020; the full record is held by the Sarawak Tropical Peat Research Institute. | FLUXNET site metadata: 1.4536, 111.1495, AsiaFlux, EBF. C7 (Aeries 2023) has 2011-2015 water-table loggers in the same national park. | Daily WT for this forest for 2011-2014 is public on figshare (doi:10.6084/m9.figshare.25299358) and half-hourly WT for Nov-Dec 2013 on Zenodo (doi:10.5281/zenodo.1161966); see EXPANDED_2006-2026 rows A15-A16.</t>
         </is>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Two Zenodo versions are kept: data/ holds 7500659 (the index link), data/zenodo_7728463_v03/ the version the paper cites. The daily GWL series is identical in both; v03 expands the diel ET panels of ED Fig. 2. | Only the intact-site GWL is published as a daily series; plantation and degraded-site GWL appear only as annual means (ED Table 2 in the paper). | Fig. 1 file gives the Acacia tower at 0 30'57"N, 102 02'11"E, about 70 km west of the other towers although the paper describes one landscape; check against the paper's Fig. 1 before using it.</t>
+          <t>Two Zenodo versions are kept: data/ holds 7500659 (the index link), data/zenodo_7728463_v03/ the version the paper cites. The daily GWL series is identical in both; v03 expands the diel ET panels of ED Fig. 2. | Only the intact-site GWL is published as a daily series; plantation and degraded-site GWL appear only as annual means (ED Table 2 in the paper). | Fig. 1 file gives the Acacia tower at 0 30'57"N, 102 02'11"E, about 70 km west of the other towers; Deshmukh et al. 2020 (GCB, doi:10.1111/gcb.15019) gives the same position, so the coordinate is correct.</t>
         </is>
       </c>
     </row>
@@ -7468,7 +7468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7634,73 +7634,73 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A8</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Acacia tower coordinate</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>A/B</t>
+          <t>(not given)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Not downloadable: Exeter files embargoed, paper says 'on request'</t>
+          <t>0.5159 N, 102.0364 E; confirmed by Deshmukh et al. 2020</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>A13-14</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Paper behind the CIFOR DOI</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Swails 2019</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>DATA.00061 is the replication data of Hergoualc'h et al. 2017</t>
+          <t>Not downloadable: Exeter files embargoed, paper says 'on request'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>A13-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Paper behind the CIFOR DOI</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>C (figures only)</t>
+          <t>Swails 2019</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Zenodo 10427000 (CC-BY) has manual water depth per chamber visit; hourly logger data not archived</t>
+          <t>DATA.00061 is the replication data of Hergoualc'h et al. 2017</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>C8-9</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -7715,56 +7715,78 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Ledger 2023 supplement has manual and logger water tables and site coordinates</t>
+          <t>Zenodo 10427000 (CC-BY) has manual water depth per chamber visit; hourly logger data not archived</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C10-11</t>
+          <t>C8-9</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Central Kalimantan, South Sumatra</t>
+          <t>C (figures only)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Central Kalimantan only</t>
+          <t>Ledger 2023 supplement has manual and logger water tables and site coordinates</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>C10-11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Central Kalimantan, South Sumatra</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Central Kalimantan only</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Resolution</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Daily, ~25 y</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Download holds 10 summary GeoTIFFs (0.1 deg, 2000-2024); daily series only on request</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>